<commit_message>
docs(pe4): completar seccion 4 - correcciones aplicadas a defectos criticos y mayores
</commit_message>
<xml_diff>
--- a/02_Inspeccion/AnexoB_registro_defectos.xlsx
+++ b/02_Inspeccion/AnexoB_registro_defectos.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Andy Mendoza\Desktop\files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Andy Mendoza\Music\ISR401-PFC-ERS-EQUIPOB\02_Inspeccion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6754B9F-562E-4C1E-80BA-C95E658F5BB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F99E8B6-4102-4B70-9BEB-0C1D23D4F574}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -113,9 +113,6 @@
     <t>Winston Cedeño</t>
   </si>
   <si>
-    <t>No</t>
-  </si>
-  <si>
     <t>3.2.12 (RF-12) y 4.2 (CU-09)</t>
   </si>
   <si>
@@ -312,6 +309,9 @@
   </si>
   <si>
     <t>Sección 5.5 completa</t>
+  </si>
+  <si>
+    <t>Si</t>
   </si>
 </sst>
 </file>
@@ -778,7 +778,7 @@
         <v>5</v>
       </c>
       <c r="B5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>6</v>
@@ -850,7 +850,7 @@
         <v>24</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>25</v>
+        <v>91</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="54.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -858,25 +858,25 @@
         <v>2</v>
       </c>
       <c r="B10" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C10" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="D10" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="E10" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="E10" s="6" t="s">
+      <c r="F10" s="4" t="s">
         <v>29</v>
-      </c>
-      <c r="F10" s="4" t="s">
-        <v>30</v>
       </c>
       <c r="G10" s="3" t="s">
         <v>24</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>25</v>
+        <v>91</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="54.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -884,25 +884,25 @@
         <v>3</v>
       </c>
       <c r="B11" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C11" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="D11" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="D11" s="3" t="s">
+      <c r="E11" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="F11" s="4" t="s">
         <v>33</v>
-      </c>
-      <c r="E11" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="F11" s="4" t="s">
-        <v>34</v>
       </c>
       <c r="G11" s="3" t="s">
         <v>24</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>25</v>
+        <v>91</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="54.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -910,25 +910,25 @@
         <v>4</v>
       </c>
       <c r="B12" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C12" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="D12" s="3" t="s">
         <v>36</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>37</v>
       </c>
       <c r="E12" s="5" t="s">
         <v>22</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="G12" s="3" t="s">
         <v>24</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>25</v>
+        <v>91</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="54.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -936,25 +936,25 @@
         <v>5</v>
       </c>
       <c r="B13" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C13" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="D13" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="E13" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="E13" s="7" t="s">
+      <c r="F13" s="4" t="s">
         <v>42</v>
-      </c>
-      <c r="F13" s="4" t="s">
-        <v>43</v>
       </c>
       <c r="G13" s="3" t="s">
         <v>24</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>25</v>
+        <v>91</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="54.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -962,25 +962,25 @@
         <v>6</v>
       </c>
       <c r="B14" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C14" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="D14" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="D14" s="3" t="s">
+      <c r="E14" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="F14" s="4" t="s">
         <v>46</v>
-      </c>
-      <c r="E14" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="F14" s="4" t="s">
-        <v>47</v>
       </c>
       <c r="G14" s="3" t="s">
         <v>24</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>25</v>
+        <v>91</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="54.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -988,10 +988,10 @@
         <v>7</v>
       </c>
       <c r="B15" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C15" s="4" t="s">
         <v>48</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>49</v>
       </c>
       <c r="D15" s="3" t="s">
         <v>21</v>
@@ -1000,13 +1000,13 @@
         <v>22</v>
       </c>
       <c r="F15" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="G15" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="G15" s="3" t="s">
-        <v>51</v>
-      </c>
       <c r="H15" s="3" t="s">
-        <v>25</v>
+        <v>91</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="54.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1014,10 +1014,10 @@
         <v>8</v>
       </c>
       <c r="B16" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C16" s="4" t="s">
         <v>52</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>53</v>
       </c>
       <c r="D16" s="3" t="s">
         <v>21</v>
@@ -1026,13 +1026,13 @@
         <v>22</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>25</v>
+        <v>91</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="54.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1040,25 +1040,25 @@
         <v>9</v>
       </c>
       <c r="B17" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="C17" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="D17" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E17" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="F17" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="D17" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="E17" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="F17" s="4" t="s">
-        <v>57</v>
-      </c>
       <c r="G17" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>25</v>
+        <v>91</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="54.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1066,25 +1066,25 @@
         <v>10</v>
       </c>
       <c r="B18" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="C18" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="C18" s="4" t="s">
+      <c r="D18" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E18" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="F18" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="D18" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="E18" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="F18" s="4" t="s">
-        <v>60</v>
-      </c>
       <c r="G18" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H18" s="3" t="s">
-        <v>25</v>
+        <v>91</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="54.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1092,25 +1092,25 @@
         <v>11</v>
       </c>
       <c r="B19" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C19" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="C19" s="4" t="s">
-        <v>62</v>
-      </c>
       <c r="D19" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E19" s="5" t="s">
         <v>22</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>25</v>
+        <v>91</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="54.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1118,25 +1118,25 @@
         <v>12</v>
       </c>
       <c r="B20" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="C20" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="C20" s="4" t="s">
-        <v>65</v>
-      </c>
       <c r="D20" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E20" s="5" t="s">
         <v>22</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H20" s="3" t="s">
-        <v>25</v>
+        <v>91</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="54.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1144,25 +1144,25 @@
         <v>13</v>
       </c>
       <c r="B21" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="C21" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="C21" s="4" t="s">
+      <c r="D21" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="F21" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="D21" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="E21" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="F21" s="4" t="s">
-        <v>90</v>
-      </c>
       <c r="G21" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="H21" s="3" t="s">
-        <v>25</v>
+        <v>91</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="54.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1170,25 +1170,25 @@
         <v>14</v>
       </c>
       <c r="B22" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="C22" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="C22" s="4" t="s">
-        <v>69</v>
-      </c>
       <c r="D22" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E22" s="5" t="s">
         <v>22</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="H22" s="3" t="s">
-        <v>25</v>
+        <v>91</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="54.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1196,25 +1196,25 @@
         <v>15</v>
       </c>
       <c r="B23" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C23" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="C23" s="4" t="s">
+      <c r="D23" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="E23" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="F23" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="D23" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="E23" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="F23" s="4" t="s">
-        <v>72</v>
-      </c>
       <c r="G23" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="H23" s="3" t="s">
-        <v>25</v>
+        <v>91</v>
       </c>
     </row>
     <row r="24" spans="1:8" ht="54.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1222,25 +1222,25 @@
         <v>16</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E24" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="G24" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="H24" s="3" t="s">
-        <v>25</v>
+        <v>91</v>
       </c>
     </row>
     <row r="25" spans="1:8" ht="54.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1248,25 +1248,25 @@
         <v>17</v>
       </c>
       <c r="B25" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="C25" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="C25" s="4" t="s">
-        <v>75</v>
-      </c>
       <c r="D25" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E25" s="5" t="s">
         <v>22</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>25</v>
+        <v>91</v>
       </c>
     </row>
     <row r="26" spans="1:8" ht="54.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1274,30 +1274,30 @@
         <v>18</v>
       </c>
       <c r="B26" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="C26" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="C26" s="4" t="s">
-        <v>77</v>
-      </c>
       <c r="D26" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E26" s="5" t="s">
         <v>22</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="G26" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="H26" s="3" t="s">
-        <v>25</v>
+        <v>91</v>
       </c>
     </row>
     <row r="28" spans="1:8" ht="10.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="12" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B28" s="12"/>
       <c r="C28" s="12"/>
@@ -1309,26 +1309,26 @@
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A31" s="8" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B31">
         <f>COUNTIF(E9:E26,"Crítico")</f>
         <v>2</v>
       </c>
       <c r="C31" s="8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D31">
         <f>COUNTIF(E9:E26,"Mayor")</f>
         <v>7</v>
       </c>
       <c r="E31" s="8" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F31">
         <f>COUNTIF(E9:E26,"Menor")</f>
@@ -1337,7 +1337,7 @@
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B32">
         <f>COUNTA(C9:C26)</f>
@@ -1346,7 +1346,7 @@
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D33">
         <f>COUNTIF(E9:E26,"Crítico")+COUNTIF(E9:E26,"Mayor")</f>

</xml_diff>